<commit_message>
Improve newsroom presentation and demo content
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,23 +482,29 @@
           <t>status</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>featured</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>is_demo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>beispiel-001</t>
+          <t>demo-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Beispielzeile entfernen</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
+          <t>Demo: Wie sich Frankfurt im Blick behalten laesst</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
@@ -507,20 +513,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Beispieltext durch eine gepruefte Meldung ersetzen.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Beispielmeldung zur Darstellung des Newsrooms. Vor dem Livegang durch eine recherchierte Meldung ersetzen.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Dies ist kein aktueller Nachrichtenbericht. Die Zeile zeigt, wie Fakten, Einordnung und Quelle spaeter auf der Website erscheinen.</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Quelle eintragen</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://example.com</t>
-        </is>
-      </c>
+          <t>DEMO-INHALT</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>mittel</t>
@@ -529,12 +535,144 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Beispielbild</t>
+          <t>Demo-Inhalt</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>demo-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Demo: Ein Special Movement sachlich einordnen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Special Movement</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beispiel fuer eine klar gekennzeichnete Meldung ohne Spekulationen oder unbestaetigte Ursachen.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Nur bestaetigte Angaben wuerden im echten Betrieb veroeffentlicht. Externe Trackingdaten waeren dabei niemals die einzige Quelle.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>DEMO-INHALT</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Demo-Inhalt</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>demo-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Demo: Infrastruktur am Flughafen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Terminal 3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Beispiel fuer ein dauerhaft relevantes Hintergrundthema rund um Frankfurt Airport.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Evergreen-Inhalte koennen an nachrichtenarmen Tagen genutzt werden, wenn sie quellenbasiert erstellt und korrekt belegt sind.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>DEMO-INHALT</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Demo-Inhalt</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand AeroNewsFRA editorial website
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,8 +504,6 @@
           <t>Demo: Wie sich Frankfurt im Blick behalten laesst</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Frankfurt Airport</t>
@@ -526,13 +524,11 @@
           <t>DEMO-INHALT</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>mittel</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>Demo-Inhalt</t>
@@ -565,8 +561,6 @@
           <t>Demo: Ein Special Movement sachlich einordnen</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Special Movement</t>
@@ -587,13 +581,11 @@
           <t>DEMO-INHALT</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>mittel</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>Demo-Inhalt</t>
@@ -626,8 +618,6 @@
           <t>Demo: Infrastruktur am Flughafen</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Terminal 3</t>
@@ -648,13 +638,11 @@
           <t>DEMO-INHALT</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>niedrig</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>Demo-Inhalt</t>
@@ -673,6 +661,67 @@
       <c r="O4" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>incident-geruch-pruefung</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pruefung: Geruch an Bord fuehrte zur Rueckkehr nach Frankfurt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Notfall</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Redaktioneller Pruefeintrag: Der konkrete Vorfall muss vor einer Veroeffentlichung eindeutig ueber Datum, Flugnummer und belastbare Quelle zugeordnet werden.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Bis zur eindeutigen Bestaetigung bleibt dieser Eintrag unsichtbar. Keine Ursache und keine weiteren Details werden abgeleitet.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Noch zu bestaetigen</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Pruefeintrag</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace demo posts with verified FRA news
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,42 +496,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>demo-001</t>
+          <t>lh573-geruch-brazzaville</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Demo: Wie sich Frankfurt im Blick behalten laesst</t>
-        </is>
-      </c>
+          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Frankfurt Airport</t>
+          <t>Special Movement</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Beispielmeldung zur Darstellung des Newsrooms. Vor dem Livegang durch eine recherchierte Meldung ersetzen.</t>
+          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dies ist kein aktueller Nachrichtenbericht. Die Zeile zeigt, wie Fakten, Einordnung und Quelle spaeter auf der Website erscheinen.</t>
+          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DEMO-INHALT</t>
+          <t>RTL.de</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>mittel</t>
-        </is>
-      </c>
+          <t>hoch</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Demo-Inhalt</t>
+          <t>Symbolbild: Boeing 747-8</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -546,49 +558,61 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>demo-002</t>
+          <t>fraport-juli-traffic</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Demo: Ein Special Movement sachlich einordnen</t>
-        </is>
-      </c>
+          <t>Frankfurt Airport erreicht im Juli rund 6,2 Millionen Passagiere</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Special Movement</t>
+          <t>Frankfurt Airport</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Beispiel fuer eine klar gekennzeichnete Meldung ohne Spekulationen oder unbestaetigte Ursachen.</t>
+          <t>Die Passagierzahl am Flughafen Frankfurt lag im Juli 2026 rund 1,4 Prozent über dem Vorjahresmonat.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Nur bestaetigte Angaben wuerden im echten Betrieb veroeffentlicht. Externe Trackingdaten waeren dabei niemals die einzige Quelle.</t>
+          <t>Nach den veröffentlichten Verkehrszahlen wurden im Juli rund 6,2 Millionen Passagiere gezählt. Gleichzeitig gingen die Flugbewegungen um 3,2 Prozent auf 41.286 Starts und Landungen zurück. Das Cargo-Aufkommen stieg um 0,9 Prozent auf 180.622 Tonnen.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DEMO-INHALT</t>
+          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://payloadasia.com/2026/08/fraport-reports-july-growth-frankfurt-passenger-traffic-cargo-volumes/</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>mittel</t>
-        </is>
-      </c>
+          <t>hoch</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Demo-Inhalt</t>
+          <t>Flughafen Frankfurt: Verkehrszahlen Juli 2026</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -603,49 +627,61 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>demo-003</t>
+          <t>fraport-h1-traffic</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Demo: Infrastruktur am Flughafen</t>
-        </is>
-      </c>
+          <t>Fraport hält Jahresausblick trotz schwächerem ersten Halbjahr</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Terminal 3</t>
+          <t>Verkehrszahlen</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Beispiel fuer ein dauerhaft relevantes Hintergrundthema rund um Frankfurt Airport.</t>
+          <t>Im ersten Halbjahr 2026 nutzten rund 28,9 Millionen Passagiere den Flughafen Frankfurt, 0,8 Prozent weniger als im Vorjahreszeitraum.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Evergreen-Inhalte koennen an nachrichtenarmen Tagen genutzt werden, wenn sie quellenbasiert erstellt und korrekt belegt sind.</t>
+          <t>Fraport führte die Entwicklung unter anderem auf Streiks bei Lufthansa und die geringere Nachfrage nach Verbindungen in den Nahen Osten zurück. Für das Gesamtjahr erwartet Fraport am Standort Frankfurt ungefähr das Passagierniveau von 2025. Die Angaben stammen aus der veröffentlichten Halbjahresauswertung.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DEMO-INHALT</t>
+          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://payloadasia.com/2026/07/fraport-maintains-2026-outlook-frankfurt-traffic-softens-first-half/</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>niedrig</t>
-        </is>
-      </c>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Demo-Inhalt</t>
+          <t>Fraport Halbjahresauswertung 2026</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -659,67 +695,6 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>incident-geruch-pruefung</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pruefung: Geruch an Bord fuehrte zur Rueckkehr nach Frankfurt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Notfall</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Redaktioneller Pruefeintrag: Der konkrete Vorfall muss vor einer Veroeffentlichung eindeutig ueber Datum, Flugnummer und belastbare Quelle zugeordnet werden.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Bis zur eindeutigen Bestaetigung bleibt dieser Eintrag unsichtbar. Keine Ursache und keine weiteren Details werden abgeleitet.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Noch zu bestaetigen</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>mittel</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Pruefeintrag</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>

<commit_message>
Add daily research and review workflow
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -496,43 +496,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lh573-geruch-brazzaville</t>
+          <t>fraport-juli-traffic</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
+          <t>Frankfurt Airport erreicht im Juli rund 6,2 Millionen Passagiere</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Special Movement</t>
+          <t>Frankfurt Airport</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
+          <t>Die Passagierzahl am Flughafen Frankfurt lag im Juli 2026 rund 1,4 Prozent über dem Vorjahresmonat.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
+          <t>Nach den veröffentlichten Verkehrszahlen wurden im Juli rund 6,2 Millionen Passagiere gezählt. Gleichzeitig gingen die Flugbewegungen um 3,2 Prozent auf 41.286 Starts und Landungen zurück. Das Cargo-Aufkommen stieg um 0,9 Prozent auf 180.622 Tonnen.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>RTL.de</t>
+          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
+          <t>https://payloadasia.com/2026/08/fraport-reports-july-growth-frankfurt-passenger-traffic-cargo-volumes/</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -543,7 +543,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Symbolbild: Boeing 747-8</t>
+          <t>Flughafen Frankfurt: Verkehrszahlen Juli 2026</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -565,43 +565,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fraport-juli-traffic</t>
+          <t>lh573-geruch-brazzaville</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Frankfurt Airport erreicht im Juli rund 6,2 Millionen Passagiere</t>
+          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Frankfurt Airport</t>
+          <t>Special Movement</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Die Passagierzahl am Flughafen Frankfurt lag im Juli 2026 rund 1,4 Prozent über dem Vorjahresmonat.</t>
+          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Nach den veröffentlichten Verkehrszahlen wurden im Juli rund 6,2 Millionen Passagiere gezählt. Gleichzeitig gingen die Flugbewegungen um 3,2 Prozent auf 41.286 Starts und Landungen zurück. Das Cargo-Aufkommen stieg um 0,9 Prozent auf 180.622 Tonnen.</t>
+          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
+          <t>RTL.de</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://payloadasia.com/2026/08/fraport-reports-july-growth-frankfurt-passenger-traffic-cargo-volumes/</t>
+          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flughafen Frankfurt: Verkehrszahlen Juli 2026</t>
+          <t>Symbolbild: Boeing 747-8</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">

</xml_diff>

<commit_message>
Publish verified daily FRA news
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,43 +565,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lh573-geruch-brazzaville</t>
+          <t>auto-dae28e3b4373</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
+          <t>Deutlich weniger Flüge am Frankfurter Flughafen</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Special Movement</t>
+          <t>Frankfurt Airport</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
+          <t>Im Juli 2026 wurden am Flughafen Frankfurt rund 6,2 Millionen Passagiere gezählt, obwohl die Zahl der Starts und Landungen zurückging.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
+          <t>Nach den von Fraport veröffentlichten und von aero.de zusammengefassten Zahlen sanken die Flugbewegungen um 3,2 Prozent auf 41.286. Die Passagierzahl stieg dagegen um 1,4 Prozent. Als Gründe werden eine höhere Auslastung und der Einsatz größerer Flugzeuge genannt.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RTL.de</t>
+          <t>aero.de</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
+          <t>https://www.aero.de/news-53366/Deutlich-weniger-Fluege-am-Frankfurter-Flughafen.html</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -610,11 +610,7 @@
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Symbolbild: Boeing 747-8</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>published</t>
@@ -622,7 +618,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -634,67 +630,266 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fraport-h1-traffic</t>
+          <t>auto-6a58b9d3aef5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fraport hält Jahresausblick trotz schwächerem ersten Halbjahr</t>
+          <t>Wachstum bei Lufthansa City Airlines geht trotz Schlichtung weiter</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
+          <t>Airlines</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Lufthansa City Airlines soll ihr Flottenwachstum trotz der Schlichtungsvereinbarung zwischen Lufthansa und der Vereinigung Cockpit fortsetzen können.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>aeroTELEGRAPH berichtet unter Berufung auf eine Mitteilung der Gewerkschaft Verdi, dass neue Flugzeuge und Wechsel aus dem Lufthansa-AOC weiterhin möglich sein sollen. Ein direkter operativer Effekt für Frankfurt ist in der Meldung nicht genannt; der Beitrag wird deshalb als mittel relevant eingeordnet.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>aeroTELEGRAPH</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.aerotelegraph.com/ticker/wachstum-bei-lufthansa-city-airlines-geht-trotz-schlichtung-weiter/kbrvm52</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>auto-e37a0f8cf765</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lufthansa und Vereinigung Cockpit vereinbaren Schlichtung</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Airlines</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Lufthansa und die Vereinigung Cockpit haben eine Vereinbarung für Schlichtung und Mediation offener Tarifthemen getroffen.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Laut aero.de sollen die Schlichtungen möglicherweise noch im August beginnen. Ein Abschluss des Gesamtverfahrens ist bis Ende Dezember 2026 vorgesehen. Die Meldung ist für Frankfurt relevant, weil Lufthansa am Standort ein zentrales Drehkreuz betreibt; konkrete Auswirkungen auf den Flugbetrieb sind damit nicht automatisch verbunden.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>aero.de</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.aero.de/news-53344/Lufthansa-und-Vereinigung-Cockpit-vereinbaren-Schlichtung.html</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>lh573-geruch-brazzaville</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Special Movement</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>RTL.de</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>hoch</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Symbolbild: Boeing 747-8</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fraport-h1-traffic</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fraport hält Jahresausblick trotz schwächerem ersten Halbjahr</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Verkehrszahlen</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Im ersten Halbjahr 2026 nutzten rund 28,9 Millionen Passagiere den Flughafen Frankfurt, 0,8 Prozent weniger als im Vorjahreszeitraum.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Fraport führte die Entwicklung unter anderem auf Streiks bei Lufthansa und die geringere Nachfrage nach Verbindungen in den Nahen Osten zurück. Für das Gesamtjahr erwartet Fraport am Standort Frankfurt ungefähr das Passagierniveau von 2025. Die Angaben stammen aus der veröffentlichten Halbjahresauswertung.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>https://payloadasia.com/2026/07/fraport-maintains-2026-outlook-frankfurt-traffic-softens-first-half/</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>mittel</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>Fraport Halbjahresauswertung 2026</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>published</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>

<commit_message>
Remove duplicate traffic report
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,12 +496,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>fraport-juli-traffic</t>
+          <t>auto-dae28e3b4373</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Frankfurt Airport erreicht im Juli rund 6,2 Millionen Passagiere</t>
+          <t>Deutlich weniger Flüge am Frankfurter Flughafen</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -517,22 +517,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Die Passagierzahl am Flughafen Frankfurt lag im Juli 2026 rund 1,4 Prozent über dem Vorjahresmonat.</t>
+          <t>Im Juli 2026 wurden am Flughafen Frankfurt rund 6,2 Millionen Passagiere gezählt, obwohl die Zahl der Starts und Landungen zurückging.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Nach den veröffentlichten Verkehrszahlen wurden im Juli rund 6,2 Millionen Passagiere gezählt. Gleichzeitig gingen die Flugbewegungen um 3,2 Prozent auf 41.286 Starts und Landungen zurück. Das Cargo-Aufkommen stieg um 0,9 Prozent auf 180.622 Tonnen.</t>
+          <t>Nach den von Fraport veröffentlichten und von aero.de zusammengefassten Zahlen sanken die Flugbewegungen um 3,2 Prozent auf 41.286. Die Passagierzahl stieg dagegen um 1,4 Prozent. Als Gründe werden eine höhere Auslastung und der Einsatz größerer Flugzeuge genannt.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
+          <t>aero.de</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://payloadasia.com/2026/08/fraport-reports-july-growth-frankfurt-passenger-traffic-cargo-volumes/</t>
+          <t>https://www.aero.de/news-53366/Deutlich-weniger-Fluege-am-Frankfurter-Flughafen.html</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -541,11 +541,7 @@
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Flughafen Frankfurt: Verkehrszahlen Juli 2026</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>published</t>
@@ -553,7 +549,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -565,12 +561,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>auto-dae28e3b4373</t>
+          <t>auto-6a58b9d3aef5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Deutlich weniger Flüge am Frankfurter Flughafen</t>
+          <t>Wachstum bei Lufthansa City Airlines geht trotz Schlichtung weiter</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -581,32 +577,32 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Frankfurt Airport</t>
+          <t>Airlines</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Im Juli 2026 wurden am Flughafen Frankfurt rund 6,2 Millionen Passagiere gezählt, obwohl die Zahl der Starts und Landungen zurückging.</t>
+          <t>Lufthansa City Airlines soll ihr Flottenwachstum trotz der Schlichtungsvereinbarung zwischen Lufthansa und der Vereinigung Cockpit fortsetzen können.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Nach den von Fraport veröffentlichten und von aero.de zusammengefassten Zahlen sanken die Flugbewegungen um 3,2 Prozent auf 41.286. Die Passagierzahl stieg dagegen um 1,4 Prozent. Als Gründe werden eine höhere Auslastung und der Einsatz größerer Flugzeuge genannt.</t>
+          <t>aeroTELEGRAPH berichtet unter Berufung auf eine Mitteilung der Gewerkschaft Verdi, dass neue Flugzeuge und Wechsel aus dem Lufthansa-AOC weiterhin möglich sein sollen. Ein direkter operativer Effekt für Frankfurt ist in der Meldung nicht genannt; der Beitrag wird deshalb als mittel relevant eingeordnet.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>aero.de</t>
+          <t>aeroTELEGRAPH</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.aero.de/news-53366/Deutlich-weniger-Fluege-am-Frankfurter-Flughafen.html</t>
+          <t>https://www.aerotelegraph.com/ticker/wachstum-bei-lufthansa-city-airlines-geht-trotz-schlichtung-weiter/kbrvm52</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>hoch</t>
+          <t>mittel</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -630,17 +626,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>auto-6a58b9d3aef5</t>
+          <t>auto-e37a0f8cf765</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wachstum bei Lufthansa City Airlines geht trotz Schlichtung weiter</t>
+          <t>Lufthansa und Vereinigung Cockpit vereinbaren Schlichtung</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -651,22 +647,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Lufthansa City Airlines soll ihr Flottenwachstum trotz der Schlichtungsvereinbarung zwischen Lufthansa und der Vereinigung Cockpit fortsetzen können.</t>
+          <t>Lufthansa und die Vereinigung Cockpit haben eine Vereinbarung für Schlichtung und Mediation offener Tarifthemen getroffen.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>aeroTELEGRAPH berichtet unter Berufung auf eine Mitteilung der Gewerkschaft Verdi, dass neue Flugzeuge und Wechsel aus dem Lufthansa-AOC weiterhin möglich sein sollen. Ein direkter operativer Effekt für Frankfurt ist in der Meldung nicht genannt; der Beitrag wird deshalb als mittel relevant eingeordnet.</t>
+          <t>Laut aero.de sollen die Schlichtungen möglicherweise noch im August beginnen. Ein Abschluss des Gesamtverfahrens ist bis Ende Dezember 2026 vorgesehen. Die Meldung ist für Frankfurt relevant, weil Lufthansa am Standort ein zentrales Drehkreuz betreibt; konkrete Auswirkungen auf den Flugbetrieb sind damit nicht automatisch verbunden.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>aeroTELEGRAPH</t>
+          <t>aero.de</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.aerotelegraph.com/ticker/wachstum-bei-lufthansa-city-airlines-geht-trotz-schlichtung-weiter/kbrvm52</t>
+          <t>https://www.aero.de/news-53344/Lufthansa-und-Vereinigung-Cockpit-vereinbaren-Schlichtung.html</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -695,52 +691,56 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>auto-e37a0f8cf765</t>
+          <t>lh573-geruch-brazzaville</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lufthansa und Vereinigung Cockpit vereinbaren Schlichtung</t>
+          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Airlines</t>
+          <t>Special Movement</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Lufthansa und die Vereinigung Cockpit haben eine Vereinbarung für Schlichtung und Mediation offener Tarifthemen getroffen.</t>
+          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Laut aero.de sollen die Schlichtungen möglicherweise noch im August beginnen. Ein Abschluss des Gesamtverfahrens ist bis Ende Dezember 2026 vorgesehen. Die Meldung ist für Frankfurt relevant, weil Lufthansa am Standort ein zentrales Drehkreuz betreibt; konkrete Auswirkungen auf den Flugbetrieb sind damit nicht automatisch verbunden.</t>
+          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>aero.de</t>
+          <t>RTL.de</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.aero.de/news-53344/Lufthansa-und-Vereinigung-Cockpit-vereinbaren-Schlichtung.html</t>
+          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>mittel</t>
+          <t>hoch</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Symbolbild: Boeing 747-8</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>published</t>
@@ -748,7 +748,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -760,54 +760,54 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>lh573-geruch-brazzaville</t>
+          <t>fraport-h1-traffic</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lufthansa LH573 landet nach Geruch in der Kabine außerplanmäßig</t>
+          <t>Fraport hält Jahresausblick trotz schwächerem ersten Halbjahr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Special Movement</t>
+          <t>Verkehrszahlen</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Ein Lufthansa-Jumbo auf dem Weg von Johannesburg nach Frankfurt ist nach einem undefinierbaren Geruch in der Kabine sicher in Brazzaville zwischengelandet.</t>
+          <t>Im ersten Halbjahr 2026 nutzten rund 28,9 Millionen Passagiere den Flughafen Frankfurt, 0,8 Prozent weniger als im Vorjahreszeitraum.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lufthansa bestätigte gegenüber RTL, dass alle 363 Passagiere und die 16-köpfige Crew das Flugzeug sicher verlassen konnten. Die Boeing 747-8 blieb zunächst zur technischen Untersuchung in Brazzaville. Eine Ursache wurde in der vorliegenden Bestätigung nicht genannt.</t>
+          <t>Fraport führte die Entwicklung unter anderem auf Streiks bei Lufthansa und die geringere Nachfrage nach Verbindungen in den Nahen Osten zurück. Für das Gesamtjahr erwartet Fraport am Standort Frankfurt ungefähr das Passagierniveau von 2025. Die Angaben stammen aus der veröffentlichten Halbjahresauswertung.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>RTL.de</t>
+          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.rtl.de/news/lufthansa-flug-lh573-sendet-notsignal-boeing-747-muss-sofort-landen-id31168621.html</t>
+          <t>https://payloadasia.com/2026/07/fraport-maintains-2026-outlook-frankfurt-traffic-softens-first-half/</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>hoch</t>
+          <t>mittel</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Symbolbild: Boeing 747-8</t>
+          <t>Fraport Halbjahresauswertung 2026</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -817,79 +817,10 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>fraport-h1-traffic</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Fraport hält Jahresausblick trotz schwächerem ersten Halbjahr</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Verkehrszahlen</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Im ersten Halbjahr 2026 nutzten rund 28,9 Millionen Passagiere den Flughafen Frankfurt, 0,8 Prozent weniger als im Vorjahreszeitraum.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Fraport führte die Entwicklung unter anderem auf Streiks bei Lufthansa und die geringere Nachfrage nach Verbindungen in den Nahen Osten zurück. Für das Gesamtjahr erwartet Fraport am Standort Frankfurt ungefähr das Passagierniveau von 2025. Die Angaben stammen aus der veröffentlichten Halbjahresauswertung.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Fraport-Verkehrszahlen (berichtet von Payload Asia)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://payloadasia.com/2026/07/fraport-maintains-2026-outlook-frankfurt-traffic-softens-first-half/</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>mittel</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Fraport Halbjahresauswertung 2026</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>

<commit_message>
Stage daily FRA news candidates
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="News" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,6 @@
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Frankfurt Airport</t>
@@ -540,8 +539,6 @@
           <t>hoch</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>published</t>
@@ -574,7 +571,6 @@
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Airlines</t>
@@ -605,8 +601,6 @@
           <t>mittel</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>published</t>
@@ -639,7 +633,6 @@
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Airlines</t>
@@ -670,8 +663,6 @@
           <t>mittel</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>published</t>
@@ -704,7 +695,6 @@
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Special Movement</t>
@@ -735,7 +725,6 @@
           <t>hoch</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>Symbolbild: Boeing 747-8</t>
@@ -773,7 +762,6 @@
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Verkehrszahlen</t>
@@ -804,7 +792,6 @@
           <t>mittel</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>Fraport Halbjahresauswertung 2026</t>
@@ -821,6 +808,1306 @@
         </is>
       </c>
       <c r="O6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>auto-db4bf840d1fc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Air France pausiert Paris - Salvador im Frühjahr 2027</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Air France setzt ihre Nonstopverbindung zwischen Salvador da Bahia und Paris im Frühjahr 2027 vorübergehend aus. Zwischen dem 8. März und 22. Mai finden keine Direktflüge statt. Ab dem 24. Mai soll die Strecke wieder regulär bedient werden. Als Grund nennt Air France operative Gründe, wie das Portal Bahia Economica berichtet. Bereits gebuchte Passagiere werden während der Unterbrechung auf Gol-Flüge über São Paulo umgebucht.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>aeroTELEGRAPH</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.aerotelegraph.com/ticker/air-france-pausiert-paris-salvador-im-fruehjahr-2027/pmlsbbx</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>auto-463f30dc5cb7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Europas Kerosinkrise: Warum der Engpass bisher ausblieb – und das Risiko bleibt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>m Frühjahr schien ein Kerosinengpass unausweichlich: Straße von Hormuz blockiert, Lagerbestände niedrig, Nachfrage steigend. Doch der Markt reagierte erstaunlich schnell und zusätzliche Lieferungen aus den USA und Nigeria schlossen einen Großteil der Lücke. Entwarnung wäre trotzdem verfrüht.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>aeroTELEGRAPH</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.aerotelegraph.com/kolumnen/europas-kerosinkrise-warum-der-engpass-bisher-ausblieb-und-das-risiko-bleibt/mgx9tmm</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>auto-526e6aab2205</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Airbus A350F: Erstauslieferung doch erst 2028?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AMSTERDAM - Der neue Airbus-Frachter A350F nimmt nach Planungen des Herstellers noch 2026 ein straffes Flugtestprogramm auf. Airbus arbeitet auf ein EIS Ende 2027 hin - und will A350F ab 2028 "in bedeutenden Stückzahlen" ausliefern. Nach einem Bericht droht dem Programm eine Verzögerung.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>aero.de</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.aero.de/news-53367/Airbus-A350F-Erstauslieferung-doch-erst-2028.html</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>auto-ac0ef1288e45</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Verdi sticht Detail aus Lufthansa-Schlichtung durch</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FRANKFURT - Lufthansa stoppt für eine Schlichtung mit der Vereinigung Cockpit die Flottenerosion in der Mainline. Die Entscheidung verzögert den laufenden Ausbau von Lufthansa City Airlines aber nicht - sagt Verdi. Lufthansa kann nach Lesart der Gewerkschaft weiterhin Lufthansa-Flugzeuge zu City Airlines rüberschieben.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>aero.de</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.aero.de/news-53368/Verdi-sticht-Detail-aus-Lufthansa-Schlichtung-durch.html</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>auto-2a6324861234</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>"Weiteres Schrumpfen ist nicht in unserem Interesse"</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FRANKFURT - Schlichtung zu Betriebsrenten, vorgezogene Vergütungsverhandlungen - und eine Mediation: Lufthansa und die Vereinigung Cockpit bohren im Spätsommer die dicken Bretter. Personalvorstand Dr. Michael Niggemann spricht im Interview über die Systematik, Themenkreise - und Ziele.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>aero.de</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.aero.de/news-53352/Weiteres-Schrumpfen-ist-nicht-in-unserem-Interesse.html</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>auto-7e208b1e7ade</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Lufthansa Cargo: Customs processes at Frankfurt Airport are being further digitized. - TRANSPORT - die Zeitung für den Güterverkehr</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMixgFBVV95cUxPS1FNNVRuTFdoLUUwRTFub0FwS3hvYXRTZ0FuWmVzeWVvVDEyYWx2U01wRjVWMFphUWFYZzRadXJnTDctaXdxZzY2aUw4NnluSFFNZkptQ1ZORE9oMUg1UHVWbjNkZTBsOFBHR1JZaFJZWFUyV21MbTAtNjk5OU9hUUVKNmptZkVDWmN0cVhLUUpDT1dVSWJtUmpHWXUxakZSQzgzczZ2RS1xWnhvRmc0M3NNcUR1TDhUVWR6ZEo3LUEySVRlUmc?oc=5" target="_blank"&gt;Lufthansa Cargo: Customs processes at Frankfurt Airport are being further digitized.&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;TRANSPORT - die Zeitung für den Güterverkehr&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPS1FNNVRuTFdoLUUwRTFub0FwS3hvYXRTZ0FuWmVzeWVvVDEyYWx2U01wRjVWMFphUWFYZzRadXJnTDctaXdxZzY2aUw4NnluSFFNZkptQ1ZORE9oMUg1UHVWbjNkZTBsOFBHR1JZaFJZWFUyV21MbTAtNjk5OU9hUUVKNmptZkVDWmN0cVhLUUpDT1dVSWJtUmpHWXUxakZSQzgzczZ2RS1xWnhvRmc0M3NNcUR1TDhUVWR6ZEo3LUEySVRlUmc?oc=5</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>auto-fdb1c2e6580e</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Vietnam Airlines zieht ins Terminal 3 am Frankfurt Airport - Austrian Wings</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMinwFBVV95cUxQb2w4SXlpenNNRUFMaEpFMHFzV2psM0ktQ3lhSjVwazhLUUxOU0wtOFhEci1tQVpuaG5vWWpHMlloT0lOVWkxeDB0dFh1MnlIcFN2ajVJTFNIOG1ocHRGb3I5aFpDc2RZS2NvSzFEYjgzOTUtRlJGOG5yRWlLMUtlYlVuUTBYNEVGRXIyU3dGUjdDNjAzSFBzMmNoSUgtWnM?oc=5" target="_blank"&gt;Vietnam Airlines zieht ins Terminal 3 am Frankfurt Airport&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Austrian Wings&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQb2w4SXlpenNNRUFMaEpFMHFzV2psM0ktQ3lhSjVwazhLUUxOU0wtOFhEci1tQVpuaG5vWWpHMlloT0lOVWkxeDB0dFh1MnlIcFN2ajVJTFNIOG1ocHRGb3I5aFpDc2RZS2NvSzFEYjgzOTUtRlJGOG5yRWlLMUtlYlVuUTBYNEVGRXIyU3dGUjdDNjAzSFBzMmNoSUgtWnM?oc=5</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>auto-4df725a00fde</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Frankfurt Terminal 3 – Airlines, Lounges &amp; Anreise im Überblick - meilenoptimieren</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMibEFVX3lxTE13M0J0OTBpYXJHeU1ERmNxRUxvY3JZZC03M2dJSXNuUWMySnY2cjhzcDVlWllBbW1PRDBiT1kyNVdMRW0yY09yNkdQYTVheUh5cnozV3lES01WMWJIZFN2QnVjZTRqMDlKMXRfaQ?oc=5" target="_blank"&gt;Frankfurt Terminal 3 – Airlines, Lounges &amp; Anreise im Überblick&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;meilenoptimieren&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE13M0J0OTBpYXJHeU1ERmNxRUxvY3JZZC03M2dJSXNuUWMySnY2cjhzcDVlWllBbW1PRDBiT1kyNVdMRW0yY09yNkdQYTVheUh5cnozV3lES01WMWJIZFN2QnVjZTRqMDlKMXRfaQ?oc=5</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>auto-889aa2431620</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Terminal 3 am Flughafen Frankfurt: Alles über Airlines, Umstiege, Anfahrt - hessenschau.de</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMi4wFBVV95cUxNZk9WOEpkMW9uSUp4MjctenhRYjFSTEdzdkVIMXpDWUNPVGpscEJjLXAxQ0sxcHZUVFJCM1o5RUJxaFpZWXdGNC1COHh2Snl2NjdNbnUxa0dOYXNnLVFRNm9PYmZjLVZYVHNWZW52MXc4YVIwT19qYzBHdWRqUVR5UjZ1dWlkb2s4OE93VERyRFZ3SnB4SjM3a0xmLW5Sb3hrUi0xQk55MTVGazlhbVpwTFhUckdHVFNCdzNVdzk1dEFMeE1qdUc5TnptVlF5YzM2WW5VZnJ4NUh0Q1NseWpyS1RNMA?oc=5" target="_blank"&gt;Terminal 3 am Flughafen Frankfurt: Alles über Airlines, Umstiege, Anfahrt&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;hessenschau.de&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNZk9WOEpkMW9uSUp4MjctenhRYjFSTEdzdkVIMXpDWUNPVGpscEJjLXAxQ0sxcHZUVFJCM1o5RUJxaFpZWXdGNC1COHh2Snl2NjdNbnUxa0dOYXNnLVFRNm9PYmZjLVZYVHNWZW52MXc4YVIwT19qYzBHdWRqUVR5UjZ1dWlkb2s4OE93VERyRFZ3SnB4SjM3a0xmLW5Sb3hrUi0xQk55MTVGazlhbVpwTFhUckdHVFNCdzNVdzk1dEFMeE1qdUc5TnptVlF5YzM2WW5VZnJ4NUh0Q1NseWpyS1RNMA?oc=5</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>auto-ed08e08b238f</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Air France und KLM umgezogen - Flughafen Frankfurt schließt T2 - aeroTELEGRAPH</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMiqgFBVV95cUxNUzJBZ2duWTN3Y0FEX0ZZdldwa2lyVUpJRGVjUTNrTUtGenQtLTFaLTh6Q1ZPa0tvYTdKX2VyWXBDTkNBeVFjZmwtcXJYVmgtSktmc3poNFlZSksxaUZVVGQwZTdEdmNrVEM3Q3lvWEdmUFppT09pM0lKS3hUaWJ0RjkzMzVZdXFsUUJnajllZUNPRHNndWtsQS13QTFrVkZXdXJOa2VuTnJRZw?oc=5" target="_blank"&gt;Air France und KLM umgezogen - Flughafen Frankfurt schließt T2&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;aeroTELEGRAPH&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNUzJBZ2duWTN3Y0FEX0ZZdldwa2lyVUpJRGVjUTNrTUtGenQtLTFaLTh6Q1ZPa0tvYTdKX2VyWXBDTkNBeVFjZmwtcXJYVmgtSktmc3poNFlZSksxaUZVVGQwZTdEdmNrVEM3Q3lvWEdmUFppT09pM0lKS3hUaWJ0RjkzMzVZdXFsUUJnajllZUNPRHNndWtsQS13QTFrVkZXdXJOa2VuTnJRZw?oc=5</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>auto-b791912ff9e4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport: Auch Air France und KLM wechseln ins Terminal 3 - fvw|TravelTalk</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMirgFBVV95cUxQQTFhWTBKV3VOem9OdGYtWXJ1SURoRG0zUHpyV3p3OWJtRXNVZUJIOVVrczgzcGQxSFpUZmIweTA4SkVMVlEzZmxpS2V1RURhZE90YUVzaDlOUTVtcy1EVXFCZ3NfUDVBNnlEOWFyTXBEdGdSamFUSlUzcUF4VmstZUd5RFFDZUhPWVBXcXBZRmNtWGprSU9zbW1ldVlSeE1JeG5OX0lKVWlJMlA4aVE?oc=5" target="_blank"&gt;Frankfurt Airport: Auch Air France und KLM wechseln ins Terminal 3&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;fvw|TravelTalk&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQQTFhWTBKV3VOem9OdGYtWXJ1SURoRG0zUHpyV3p3OWJtRXNVZUJIOVVrczgzcGQxSFpUZmIweTA4SkVMVlEzZmxpS2V1RURhZE90YUVzaDlOUTVtcy1EVXFCZ3NfUDVBNnlEOWFyTXBEdGdSamFUSlUzcUF4VmstZUd5RFFDZUhPWVBXcXBZRmNtWGprSU9zbW1ldVlSeE1JeG5OX0lKVWlJMlA4aVE?oc=5</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>auto-16614984fb1d</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Flughafen Frankfurt: Aufgepasst – diese Airlines fliegen seit dem 5. Mai am neuen Terminal 3 ab - Main-Post</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMi0gFBVV95cUxNVXdldWdGLTlRcVNYakFHTVdiV1l2QXIyNkR4bDJEX21GWHc0c3BYczV6S3I2VWRScXNYTGVLdU45MXhtN3FjZUNxbERlTHYxWGZCaVlNelE3OUFNU3BHQVFCYXEtRUdMMW1MUFdtZFZGY05teUVSaFkxUm9fdEZsN3BoeEhUdFVVcUd3dEcwUHBmbWxEcER2ZF94N2RGNDFkVktnbEZ1cFZ2M0dBc21WQzFjRlNvMF96ZGYzUUZzRDk1LWtOOXVLWWl4bTRRYXB2Wnc?oc=5" target="_blank"&gt;Flughafen Frankfurt: Aufgepasst – diese Airlines fliegen seit dem 5. Mai am neuen Terminal 3 ab&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Main-Post&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNVXdldWdGLTlRcVNYakFHTVdiV1l2QXIyNkR4bDJEX21GWHc0c3BYczV6S3I2VWRScXNYTGVLdU45MXhtN3FjZUNxbERlTHYxWGZCaVlNelE3OUFNU3BHQVFCYXEtRUdMMW1MUFdtZFZGY05teUVSaFkxUm9fdEZsN3BoeEhUdFVVcUd3dEcwUHBmbWxEcER2ZF94N2RGNDFkVktnbEZ1cFZ2M0dBc21WQzFjRlNvMF96ZGYzUUZzRDk1LWtOOXVLWWl4bTRRYXB2Wnc?oc=5</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>auto-7fdf8e34c1c3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Fluggäste aufgepasst: Diese Airlines ziehen heute am Frankfurter Flughafen um - t-online – Frankfurt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMi1gFBVV95cUxNUjNzejVBeXh1RnV5cGNHNnlhUXJTb1N6MEppRXZGb1FBMHRjUHFTOTVGd2IxTlFCNUxiaGM5ZmJ5QUc4STZyQ1hEcV9sNWpFTzh6R19CNXBVTEpuTDRXNktxakRQenJ1dTVMQXRUNXE2d2NSdGhZUjBVOV9vTktaa3FUZnpuUkR4dFdqX0ItdXU3dVpmQ0kxRWFjMVhRWHVMRTRwVy1GWUdXZDNTTkdiU2praDR0SENYNVowM1ZUQWVsNkt2bmp0ak8tYWUxR0NGeEI5VzV3?oc=5" target="_blank"&gt;Fluggäste aufgepasst: Diese Airlines ziehen heute am Frankfurter Flughafen um&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;t-online – Frankfurt&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNUjNzejVBeXh1RnV5cGNHNnlhUXJTb1N6MEppRXZGb1FBMHRjUHFTOTVGd2IxTlFCNUxiaGM5ZmJ5QUc4STZyQ1hEcV9sNWpFTzh6R19CNXBVTEpuTDRXNktxakRQenJ1dTVMQXRUNXE2d2NSdGhZUjBVOV9vTktaa3FUZnpuUkR4dFdqX0ItdXU3dVpmQ0kxRWFjMVhRWHVMRTRwVy1GWUdXZDNTTkdiU2praDR0SENYNVowM1ZUQWVsNkt2bmp0ak8tYWUxR0NGeEI5VzV3?oc=5</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>auto-49937618d284</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Terminal 3 in Frankfurt eröffnet: Was Reisende jetzt wissen müssen - reisen EXCLUSIV</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMie0FVX3lxTE1NdVRoUTlZb0JIcmkwV0QtZUVPbGQ4amlGWHcwNlgzY29SRGlSd2JMam9xVjZpRzhENzRKamFoMk80eDdKdG5kLWJab2pTak9CdlliSDNkZjdER29RLWdIS0RVX3lYZU5zWWRKbGJncnZBem9mQi1zaGNWbw?oc=5" target="_blank"&gt;Terminal 3 in Frankfurt eröffnet: Was Reisende jetzt wissen müssen&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;reisen EXCLUSIV&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1NdVRoUTlZb0JIcmkwV0QtZUVPbGQ4amlGWHcwNlgzY29SRGlSd2JMam9xVjZpRzhENzRKamFoMk80eDdKdG5kLWJab2pTak9CdlliSDNkZjdER29RLWdIS0RVX3lYZU5zWWRKbGJncnZBem9mQi1zaGNWbw?oc=5</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>auto-640cee9e5121</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Terminal 3 am Flughafen Frankfurt: Fraport verrät kompletten Zeitplan für Airline-Umzüge - fnp.de</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMiswFBVV95cUxPNGp4ck0wTHo4aExLajNwOUZLSEJJNjczLXZJTXFmVjZoV1REelB4bnV3bXdybHVKeXJISUFIanIzeVhuS1dsMDhoMmhIYUJzakxaRWRpaWpXZkNhYl81WjZiYXNXRjlZTnlzUWFHdy0xbWdCaTdNM3dQRTU2X1Q2THZSVGNIaUhSNmY0Mm85UVh6TWxzQ3A0SlNraXM2T2hONXdrZ2lwUm9NUVZ4MnU5OHpMcw?oc=5" target="_blank"&gt;Terminal 3 am Flughafen Frankfurt: Fraport verrät kompletten Zeitplan für Airline-Umzüge&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;fnp.de&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPNGp4ck0wTHo4aExLajNwOUZLSEJJNjczLXZJTXFmVjZoV1REelB4bnV3bXdybHVKeXJISUFIanIzeVhuS1dsMDhoMmhIYUJzakxaRWRpaWpXZkNhYl81WjZiYXNXRjlZTnlzUWFHdy0xbWdCaTdNM3dQRTU2X1Q2THZSVGNIaUhSNmY0Mm85UVh6TWxzQ3A0SlNraXM2T2hONXdrZ2lwUm9NUVZ4MnU5OHpMcw?oc=5</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>auto-0598012a45f7</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A Milestone at FRA: the First Landing at Terminal 3 - Presseportal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMiV0FVX3lxTE5STWZuUy1NUEJwMFBjTElYYl9HRE90TU1NUEQ1YnVuVXIwQmRPaks4ZGdQUnNRS1p6WW5lZG1jVnA5QURWQm5zWTBYYkFueV9JS3J1N0xfNA?oc=5" target="_blank"&gt;A Milestone at FRA: the First Landing at Terminal 3&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Presseportal&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE5STWZuUy1NUEJwMFBjTElYYl9HRE90TU1NUEQ1YnVuVXIwQmRPaks4ZGdQUnNRS1p6WW5lZG1jVnA5QURWQm5zWTBYYkFueV9JS3J1N0xfNA?oc=5</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>auto-e35d8143da11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Neue SkyTeam Lounge im Terminal 3 Frankfurt: Zugang, Ausstattung und Einschränkungen - Frankfurtflyer.de</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMirwFBVV95cUxNOTNETUJleS1FX0dZT1FJVHBZSWtqbFhCWTNpbnBqdEl4SVcydHFDbFQyYUVwMjE0LVpKb3ZVS0FJWGIzLWxvazBiem1mYldhZnFoWVVnMS1Ea3ZTU2VOWXNkMlAwZUoxUkllaXhtbFR0OU10NURjb2JLdW9UX3U1UjZ0dExrbjFiUVZOUjVoZ21DNkxhMUQtblJ6SnlLTDBfRF9OQnVreGxUXzEyaThB?oc=5" target="_blank"&gt;Neue SkyTeam Lounge im Terminal 3 Frankfurt: Zugang, Ausstattung und Einschränkungen&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Frankfurtflyer.de&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNOTNETUJleS1FX0dZT1FJVHBZSWtqbFhCWTNpbnBqdEl4SVcydHFDbFQyYUVwMjE0LVpKb3ZVS0FJWGIzLWxvazBiem1mYldhZnFoWVVnMS1Ea3ZTU2VOWXNkMlAwZUoxUkllaXhtbFR0OU10NURjb2JLdW9UX3U1UjZ0dExrbjFiUVZOUjVoZ21DNkxhMUQtblJ6SnlLTDBfRF9OQnVreGxUXzEyaThB?oc=5</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>auto-913e97c6b478</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Kurznachrichten: Streckenstart von Edelweiss, Air Corsica, Discover Airlines und Umzug von Air France am Airport Frankfurt - Airportzentrale</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMi7gFBVV95cUxNTDY1U2VhOGVvcVp2dlcwY0gzb2hsSGFoZ1FuUWZWd2JrOGFaTjNDSFVHNTlJYS0tVW9DRDdLTElqNEtyU015emRWaVFBUXc2YUVXamM1ZW5CYzZDUjFVTlpIenBFcmVVdVNMMXZfaFZsNXBHMnIyYUJKbnhQMVBLUHJIQlVRMU8tal9UT1lLNU9XRUQtSWJKSkxpNEZTcnVVSEZMX0hlMW1EM0hEVVFBdnoxeVM1SW9XeFk4c21fRnJKc0Rwa3RhUmRnSy13U3RxdmtGUTB3bE9Db3RBRUdhNkxpNXUwZG9UOE5YRU53?oc=5" target="_blank"&gt;Kurznachrichten: Streckenstart von Edelweiss, Air Corsica, Discover Airlines und Umzug von Air France am Airport Frankfurt&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Airportzentrale&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxNTDY1U2VhOGVvcVp2dlcwY0gzb2hsSGFoZ1FuUWZWd2JrOGFaTjNDSFVHNTlJYS0tVW9DRDdLTElqNEtyU015emRWaVFBUXc2YUVXamM1ZW5CYzZDUjFVTlpIenBFcmVVdVNMMXZfaFZsNXBHMnIyYUJKbnhQMVBLUHJIQlVRMU8tal9UT1lLNU9XRUQtSWJKSkxpNEZTcnVVSEZMX0hlMW1EM0hEVVFBdnoxeVM1SW9XeFk4c21fRnJKc0Rwa3RhUmRnSy13U3RxdmtGUTB3bE9Db3RBRUdhNkxpNXUwZG9UOE5YRU53?oc=5</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>auto-b9057e59b5cb</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Flughafen Frankfurt: Korean Air wechselt in das Terminal 3 - fvw|TravelTalk</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMiowFBVV95cUxNbl9pMWZIanJOV1R1Zzc0NElHOGtwQTNVT3NXa09tSTFuQkFRZlV3T2J0bEtVQWF5cU9sUUZ5c3FfM2RCUU5oLUtFMVhoZlNiYzlRZS1wUjlFMl9QZzFINTdSbTA1S21Za1ZDbmxvZHZMZEpmYW03SDBOY1ZiUXZNQjR4cjVNcW53d19fU0VKRGFlT3hkTndpYm1UVFVKX1h2dHpJ?oc=5" target="_blank"&gt;Flughafen Frankfurt: Korean Air wechselt in das Terminal 3&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;fvw|TravelTalk&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNbl9pMWZIanJOV1R1Zzc0NElHOGtwQTNVT3NXa09tSTFuQkFRZlV3T2J0bEtVQWF5cU9sUUZ5c3FfM2RCUU5oLUtFMVhoZlNiYzlRZS1wUjlFMl9QZzFINTdSbTA1S21Za1ZDbmxvZHZMZEpmYW03SDBOY1ZiUXZNQjR4cjVNcW53d19fU0VKRGFlT3hkTndpYm1UVFVKX1h2dHpJ?oc=5</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>auto-3b4197a584d6</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Flughafen Frankfurt präsentiert Sommerflugplan - Fliegerweb</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>&lt;a href="https://news.google.com/rss/articles/CBMingFBVV95cUxNS2JnYUVJb2pJSFd2QzZCbzFWb1NCZU5rUDR4UlYtQkJENUVXenlfWUtYUkdUWTl1bzFXR2tYdW5SN19tVzJPa3EzVWtjTWZLTk5vbDFsNVBXdXE4bG5USF9pWEpQclZuZlNyZkRoSXJWUzY2ZEI2OXhHdk9aNjdUbFBUaW5UX29BN1BlVEx2SUxCUTFVY1FFVGU0dGNXQQ?oc=5" target="_blank"&gt;Flughafen Frankfurt präsentiert Sommerflugplan&lt;/a&gt;&amp;nbsp;&amp;nbsp;&lt;font color="#6f6f6f"&gt;Fliegerweb&lt;/font&gt;</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Google News FRA</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNS2JnYUVJb2pJSFd2QzZCbzFWb1NCZU5rUDR4UlYtQkJENUVXenlfWUtYUkdUWTl1bzFXR2tYdW5SN19tVzJPa3EzVWtjTWZLTk5vbDFsNVBXdXE4bG5USF9pWEpQclZuZlNyZkRoSXJWUzY2ZEI2OXhHdk9aNjdUbFBUaW5UX29BN1BlVEx2SUxCUTFVY1FFVGU0dGNXQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>